<commit_message>
Test Cases for Aarong.xlsx
</commit_message>
<xml_diff>
--- a/Test Cases for Aarong.xlsx
+++ b/Test Cases for Aarong.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bebed286a0b7e287/Documents/NEW/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{2B77E1C0-2E6C-4DBF-BCF0-3144EFCC80D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2225ED80-588F-439E-AA53-9B0E37F1563C}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="8_{2B77E1C0-2E6C-4DBF-BCF0-3144EFCC80D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AFAF4CE3-AD95-412E-AC4B-5AF18AB5F234}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="252">
   <si>
     <t xml:space="preserve">                                                                                                          Aarong Sign up</t>
   </si>
@@ -902,21 +902,6 @@
 redirect to error page</t>
   </si>
   <si>
-    <t>Verify login failed 
-thorugh facebook</t>
-  </si>
-  <si>
-    <t>Enter invalid Fb credentials.</t>
-  </si>
-  <si>
-    <t>System should show 
-an error message.</t>
-  </si>
-  <si>
-    <t>Fcaebook login button
- redirect to error page</t>
-  </si>
-  <si>
     <t>Google</t>
   </si>
   <si>
@@ -946,13 +931,19 @@
   </si>
   <si>
     <t>JIRA link</t>
+  </si>
+  <si>
+    <t>PDF</t>
+  </si>
+  <si>
+    <t>Bug Report</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1057,6 +1048,11 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1187,7 +1183,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1273,6 +1269,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1457,20 +1456,20 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>85725</xdr:rowOff>
+      <xdr:colOff>495300</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>95783</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{62A7E5D2-204B-DD89-56F0-7E5662C6EE6F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9E2F9FF4-1A81-450A-B834-EDF9BD7E57D3}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1486,8 +1485,52 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="47625"/>
-          <a:ext cx="7086600" cy="2952750"/>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7200900" cy="3820058"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>161925</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>361950</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{970B1505-4336-FE82-26F7-F9F1C9E1DCCC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="161925" y="3781425"/>
+          <a:ext cx="6905625" cy="3343275"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3007,7 +3050,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AA32"/>
+  <dimension ref="A1:AA31"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="19" customWidth="1"/>
@@ -4211,7 +4254,7 @@
     </row>
     <row r="29" spans="1:27" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A29" s="24"/>
-      <c r="B29" s="24"/>
+      <c r="B29" s="35"/>
       <c r="C29" s="7" t="s">
         <v>115</v>
       </c>
@@ -4230,8 +4273,8 @@
       <c r="H29" s="7" t="s">
         <v>240</v>
       </c>
-      <c r="I29" s="7" t="s">
-        <v>56</v>
+      <c r="I29" s="11" t="s">
+        <v>18</v>
       </c>
       <c r="J29" s="7" t="s">
         <v>15</v>
@@ -4256,27 +4299,29 @@
     </row>
     <row r="30" spans="1:27" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A30" s="24"/>
-      <c r="B30" s="25"/>
+      <c r="B30" s="30" t="s">
+        <v>241</v>
+      </c>
       <c r="C30" s="7" t="s">
         <v>119</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>242</v>
-      </c>
-      <c r="F30" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="F30" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>244</v>
+        <v>24</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>56</v>
+        <v>18</v>
       </c>
       <c r="J30" s="7" t="s">
         <v>15</v>
@@ -4300,25 +4345,23 @@
       <c r="AA30" s="16"/>
     </row>
     <row r="31" spans="1:27" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A31" s="24"/>
-      <c r="B31" s="30" t="s">
-        <v>245</v>
-      </c>
+      <c r="A31" s="25"/>
+      <c r="B31" s="25"/>
       <c r="C31" s="7" t="s">
         <v>123</v>
       </c>
       <c r="D31" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="F31" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="G31" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="E31" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="F31" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="G31" s="7" t="s">
-        <v>248</v>
-      </c>
       <c r="H31" s="7" t="s">
         <v>24</v>
       </c>
@@ -4326,69 +4369,25 @@
         <v>18</v>
       </c>
       <c r="J31" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="K31" s="16"/>
-      <c r="L31" s="16"/>
-      <c r="M31" s="16"/>
-      <c r="N31" s="16"/>
-      <c r="O31" s="16"/>
-      <c r="P31" s="16"/>
-      <c r="Q31" s="16"/>
-      <c r="R31" s="16"/>
-      <c r="S31" s="16"/>
-      <c r="T31" s="16"/>
-      <c r="U31" s="16"/>
-      <c r="V31" s="16"/>
-      <c r="W31" s="16"/>
-      <c r="X31" s="16"/>
-      <c r="Y31" s="16"/>
-      <c r="Z31" s="16"/>
-      <c r="AA31" s="16"/>
-    </row>
-    <row r="32" spans="1:27" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A32" s="25"/>
-      <c r="B32" s="25"/>
-      <c r="C32" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="D32" s="7" t="s">
-        <v>249</v>
-      </c>
-      <c r="E32" s="7" t="s">
-        <v>238</v>
-      </c>
-      <c r="F32" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="G32" s="7" t="s">
-        <v>250</v>
-      </c>
-      <c r="H32" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="I32" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="J32" s="7" t="s">
         <v>15</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="B22:B27"/>
-    <mergeCell ref="B28:B30"/>
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A4:A32"/>
+    <mergeCell ref="A4:A31"/>
     <mergeCell ref="B4:B7"/>
     <mergeCell ref="B8:B11"/>
     <mergeCell ref="B12:B15"/>
     <mergeCell ref="E13:E14"/>
     <mergeCell ref="B16:B21"/>
-    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="B28:B29"/>
   </mergeCells>
+  <phoneticPr fontId="18" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I4:I32" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I4:I31" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Pass,Fail"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4403,7 +4402,7 @@
   <sheetData>
     <row r="14" spans="16:21" x14ac:dyDescent="0.2">
       <c r="P14" s="34" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="Q14" s="34"/>
       <c r="R14" s="34"/>
@@ -4433,7 +4432,7 @@
   <sheetData>
     <row r="29" spans="17:17" x14ac:dyDescent="0.2">
       <c r="Q29" s="20" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
     </row>
   </sheetData>
@@ -4447,19 +4446,38 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B2AF56C-CEFE-412D-AAFB-5CEF6AF46D75}">
-  <dimension ref="M4"/>
+  <dimension ref="M3:M28"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="13" max="13" width="15.28515625" customWidth="1"/>
+  </cols>
   <sheetData>
+    <row r="3" spans="13:13" x14ac:dyDescent="0.2">
+      <c r="M3" t="s">
+        <v>251</v>
+      </c>
+    </row>
     <row r="4" spans="13:13" x14ac:dyDescent="0.2">
       <c r="M4" s="20" t="s">
-        <v>253</v>
+        <v>249</v>
+      </c>
+    </row>
+    <row r="27" spans="13:13" x14ac:dyDescent="0.2">
+      <c r="M27" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="28" spans="13:13" x14ac:dyDescent="0.2">
+      <c r="M28" s="20" t="s">
+        <v>250</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="M4" r:id="rId1" xr:uid="{B00154F1-3CF0-4A20-AA19-B2D96AFE5BA4}"/>
+    <hyperlink ref="M28" r:id="rId2" xr:uid="{4911641C-561B-4BF8-BEFC-8AA9CB5044FB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>